<commit_message>
experiment 1 and 2 data generation
Minor fix in the class IMPEDANCE_DATA
anova analysis of the 1st experiment
</commit_message>
<xml_diff>
--- a/data/ball_bouncing_experiment/experimental_bench_pert/data_2021_April/ball_bouncing_data.xlsx
+++ b/data/ball_bouncing_experiment/experimental_bench_pert/data_2021_April/ball_bouncing_data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fortineau_Vin\Documents\GitHub\Thesis_report\data\ball_bouncing_experiment\experimental_bench_pert\data_2021_April\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11F9E02-ED36-4944-825B-79EABFFC1FFA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1BB84E-E5B7-4F11-B9D7-CE50F7D64712}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15750" windowHeight="11775" xr2:uid="{DE8F198D-415C-4C46-986A-A987744CD0FF}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15750" windowHeight="11775" activeTab="1" xr2:uid="{DE8F198D-415C-4C46-986A-A987744CD0FF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Data summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Exp 1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$B$4:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data summary'!$B$4:$P$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="47">
   <si>
     <t>Ball bouncing performance according to the experimental conditions</t>
   </si>
@@ -151,6 +152,24 @@
   </si>
   <si>
     <t>21_apr_14</t>
+  </si>
+  <si>
+    <t>Exp Ref</t>
+  </si>
+  <si>
+    <t>exp1</t>
+  </si>
+  <si>
+    <t>Mean estim stiffness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean R^2 </t>
+  </si>
+  <si>
+    <t>Mean estim damping</t>
+  </si>
+  <si>
+    <t>Mean estim mass</t>
   </si>
 </sst>
 </file>
@@ -158,7 +177,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="00000"/>
+    <numFmt numFmtId="164" formatCode="00000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -234,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -245,13 +264,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -262,6 +278,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -576,705 +601,726 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2058B83-3B05-4319-89C1-1F726A3BB046}">
-  <dimension ref="B2:R19"/>
+  <dimension ref="B2:S19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="7.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="9" max="9" width="9" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="9" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" customWidth="1"/>
+    <col min="16" max="17" width="7.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="2:19" ht="21" x14ac:dyDescent="0.35">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:18" s="1" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="9" t="s">
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+    </row>
+    <row r="3" spans="2:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:19" s="1" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="L4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="M4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M4" s="10" t="s">
+      <c r="N4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="N4" s="10" t="s">
+      <c r="O4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="P4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="Q4" s="13"/>
+      <c r="S4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="3">
         <v>44293</v>
       </c>
-      <c r="D5" s="8">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E5" s="7">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" s="4">
         <v>0</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>314</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>275</v>
       </c>
-      <c r="K5" s="7"/>
-      <c r="L5" t="s">
+      <c r="L5" s="6"/>
+      <c r="M5" t="s">
         <v>6</v>
       </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="5">
+      <c r="N5" s="6"/>
+      <c r="O5" s="5">
         <v>0.10249999999999999</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>8.94</v>
       </c>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="3">
         <v>44293</v>
       </c>
-      <c r="D6" s="8">
+      <c r="E6" s="7">
         <v>2</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="4">
         <v>0</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>316</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>276</v>
       </c>
-      <c r="K6" s="7"/>
-      <c r="L6" t="s">
+      <c r="L6" s="6"/>
+      <c r="M6" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="7"/>
-      <c r="N6" s="5">
+      <c r="N6" s="6"/>
+      <c r="O6" s="5">
         <v>0.1885</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>28.25</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="3">
         <v>44293</v>
       </c>
-      <c r="D7" s="8">
+      <c r="E7" s="7">
         <v>3</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="4">
         <v>0</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>476</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>401</v>
       </c>
-      <c r="K7" s="7"/>
-      <c r="L7" t="s">
+      <c r="L7" s="6"/>
+      <c r="M7" t="s">
         <v>7</v>
       </c>
-      <c r="M7" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="N7" s="5">
+      <c r="N7" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="O7" s="5">
         <v>0.15590000000000001</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>33.409999999999997</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="3">
         <v>44293</v>
       </c>
-      <c r="D8" s="8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="E8" s="7">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I8" s="4">
         <v>0</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>320</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>302</v>
       </c>
-      <c r="K8" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="L8" t="s">
+      <c r="L8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M8" t="s">
         <v>6</v>
       </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="5">
+      <c r="N8" s="6"/>
+      <c r="O8" s="5">
         <v>0.1469</v>
       </c>
-      <c r="O8" s="12">
+      <c r="P8" s="11">
         <v>19.88</v>
       </c>
-      <c r="R8" t="s">
+      <c r="Q8" s="11"/>
+      <c r="S8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="3">
+      <c r="D9" s="3">
         <v>44294</v>
       </c>
-      <c r="D9" s="8">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="E9" s="7">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I9" s="4">
         <v>0.1</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>320</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>279</v>
       </c>
-      <c r="K9" s="7"/>
-      <c r="L9" t="s">
+      <c r="L9" s="6"/>
+      <c r="M9" t="s">
         <v>6</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="5">
+      <c r="N9" s="6"/>
+      <c r="O9" s="5">
         <v>0.12959999999999999</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>14.2</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="3">
+      <c r="D10" s="3">
         <v>44294</v>
       </c>
-      <c r="D10" s="8">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="E10" s="7">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="4">
+      <c r="G10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="4">
         <v>0.1</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>317</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>280</v>
       </c>
-      <c r="K10" s="7"/>
-      <c r="L10" t="s">
+      <c r="L10" s="6"/>
+      <c r="M10" t="s">
         <v>6</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="5">
+      <c r="N10" s="6"/>
+      <c r="O10" s="5">
         <v>9.2299999999999993E-2</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>7.15</v>
       </c>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="3">
         <v>44294</v>
       </c>
-      <c r="D11" s="8">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="E11" s="7">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="4">
+      <c r="G11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="4">
         <v>0.9</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>431</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>386</v>
       </c>
-      <c r="K11" s="7"/>
-      <c r="L11" t="s">
+      <c r="L11" s="6"/>
+      <c r="M11" t="s">
         <v>6</v>
       </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="5">
+      <c r="N11" s="6"/>
+      <c r="O11" s="5">
         <v>0.1221</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>16.579999999999998</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="3">
+      <c r="D12" s="3">
         <v>44294</v>
       </c>
-      <c r="D12" s="8">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="E12" s="7">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="4">
+      <c r="G12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="4">
         <v>0.9</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>398</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>362</v>
       </c>
-      <c r="K12" s="7"/>
-      <c r="L12" t="s">
+      <c r="L12" s="6"/>
+      <c r="M12" t="s">
         <v>6</v>
       </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="5">
+      <c r="N12" s="6"/>
+      <c r="O12" s="5">
         <v>0.12509999999999999</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>17.88</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="3">
+      <c r="D13" s="3">
         <v>44294</v>
       </c>
-      <c r="D13" s="8">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="E13" s="7">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="4">
+      <c r="G13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="4">
         <v>0.1</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>320</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>285</v>
       </c>
-      <c r="K13" s="7"/>
-      <c r="L13" t="s">
+      <c r="L13" s="6"/>
+      <c r="M13" t="s">
         <v>6</v>
       </c>
-      <c r="M13" s="7"/>
-      <c r="N13" s="5">
+      <c r="N13" s="6"/>
+      <c r="O13" s="5">
         <v>9.8699999999999996E-2</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>8.1</v>
       </c>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="3">
+      <c r="D14" s="3">
         <v>44294</v>
       </c>
-      <c r="D14" s="8">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="E14" s="7">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="4">
+      <c r="G14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="4">
         <v>0.9</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>351</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>327</v>
       </c>
-      <c r="K14" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="L14" t="s">
+      <c r="L14" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" t="s">
         <v>6</v>
       </c>
-      <c r="M14" s="7"/>
-      <c r="N14" s="5">
+      <c r="N14" s="6"/>
+      <c r="O14" s="5">
         <v>0.1401</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>18.89</v>
       </c>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="3">
+      <c r="D15" s="3">
         <v>44294</v>
       </c>
-      <c r="D15" s="8">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="E15" s="7">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="4">
+      <c r="G15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="4">
         <v>0.1</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>352</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>313</v>
       </c>
-      <c r="K15" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="L15" t="s">
+      <c r="L15" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M15" t="s">
         <v>6</v>
       </c>
-      <c r="M15" s="7"/>
-      <c r="N15" s="5">
+      <c r="N15" s="6"/>
+      <c r="O15" s="5">
         <v>0.10390000000000001</v>
       </c>
-      <c r="O15">
+      <c r="P15">
         <v>9.84</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="3">
+      <c r="D16" s="3">
         <v>44294</v>
       </c>
-      <c r="D16" s="8">
-        <v>1</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="E16" s="7">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G16" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I16" s="4">
         <v>0.1</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>295</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>264</v>
       </c>
-      <c r="K16" s="7"/>
-      <c r="L16" t="s">
+      <c r="L16" s="6"/>
+      <c r="M16" t="s">
         <v>7</v>
       </c>
-      <c r="M16" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="N16" s="5">
+      <c r="N16" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="O16" s="5">
         <v>0.1361</v>
       </c>
-      <c r="O16">
+      <c r="P16">
         <v>14.3</v>
       </c>
-      <c r="R16" t="s">
+      <c r="S16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="3">
+      <c r="D17" s="3">
         <v>44294</v>
       </c>
-      <c r="D17" s="8">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="E17" s="7">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I17" s="4">
         <v>0.1</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>336</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>314</v>
       </c>
-      <c r="K17" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="L17" t="s">
+      <c r="L17" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M17" t="s">
         <v>6</v>
       </c>
-      <c r="M17" s="7"/>
-      <c r="N17" s="5">
+      <c r="N17" s="6"/>
+      <c r="O17" s="5">
         <v>9.06E-2</v>
       </c>
-      <c r="O17">
+      <c r="P17">
         <v>7.5</v>
       </c>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="3">
+      <c r="D18" s="3">
         <v>44294</v>
       </c>
-      <c r="D18" s="8">
-        <v>1</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="E18" s="7">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I18" s="4">
         <v>0.1</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>312</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>287</v>
       </c>
-      <c r="K18" s="7"/>
-      <c r="L18" t="s">
+      <c r="L18" s="6"/>
+      <c r="M18" t="s">
         <v>6</v>
       </c>
-      <c r="M18" s="7"/>
-      <c r="N18" s="5">
+      <c r="N18" s="6"/>
+      <c r="O18" s="5">
         <v>9.7500000000000003E-2</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>8.2799999999999994</v>
       </c>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="3">
         <v>44295</v>
       </c>
-      <c r="D19" s="8">
-        <v>1</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="E19" s="7">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I19" s="4">
         <v>0</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>319</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>286</v>
       </c>
-      <c r="K19" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="L19" t="s">
+      <c r="L19" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M19" t="s">
         <v>6</v>
       </c>
-      <c r="M19" s="7"/>
-      <c r="N19" s="5">
+      <c r="N19" s="6"/>
+      <c r="O19" s="5">
         <v>0.12089999999999999</v>
       </c>
-      <c r="O19">
+      <c r="P19">
         <v>12.08</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:O4" xr:uid="{35B8D8CF-4A93-404A-8748-AC6A5A49E87A}"/>
+  <autoFilter ref="B4:P4" xr:uid="{35B8D8CF-4A93-404A-8748-AC6A5A49E87A}"/>
   <mergeCells count="1">
-    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B2:M2"/>
   </mergeCells>
-  <conditionalFormatting sqref="N5:N35">
+  <conditionalFormatting sqref="O5:O35">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1286,7 +1332,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O35">
+  <conditionalFormatting sqref="P5:Q35">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1301,4 +1347,274 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F6DD8F-3D3C-41CA-BBFF-93E126C20000}">
+  <dimension ref="C2:P8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="P3" s="14"/>
+    </row>
+    <row r="4" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="3">
+        <v>44293</v>
+      </c>
+      <c r="F4" s="7">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="5">
+        <v>0.10249999999999999</v>
+      </c>
+      <c r="K4">
+        <v>8.94</v>
+      </c>
+      <c r="L4" s="5">
+        <v>0.77059999999999995</v>
+      </c>
+      <c r="M4">
+        <v>340</v>
+      </c>
+      <c r="N4">
+        <v>11.6</v>
+      </c>
+      <c r="O4">
+        <v>0.53800000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="3">
+        <v>44293</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5" s="5">
+        <v>0.1885</v>
+      </c>
+      <c r="K5">
+        <v>28.25</v>
+      </c>
+      <c r="L5" s="5">
+        <v>0.77029999999999998</v>
+      </c>
+      <c r="M5">
+        <v>487</v>
+      </c>
+      <c r="N5">
+        <v>15.9</v>
+      </c>
+      <c r="O5">
+        <v>0.63700000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="3">
+        <v>44293</v>
+      </c>
+      <c r="F6" s="7">
+        <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="5">
+        <v>0.15590000000000001</v>
+      </c>
+      <c r="K6">
+        <v>33.409999999999997</v>
+      </c>
+      <c r="L6" s="5">
+        <v>0.79179999999999995</v>
+      </c>
+      <c r="M6">
+        <v>387</v>
+      </c>
+      <c r="N6">
+        <v>13.4</v>
+      </c>
+      <c r="O6">
+        <v>0.67200000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="3">
+        <v>44293</v>
+      </c>
+      <c r="F7" s="7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J7" s="5">
+        <v>0.1469</v>
+      </c>
+      <c r="K7" s="11">
+        <v>19.88</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="3">
+        <v>44295</v>
+      </c>
+      <c r="F8" s="7">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J8" s="5">
+        <v>0.12089999999999999</v>
+      </c>
+      <c r="K8">
+        <v>12.08</v>
+      </c>
+      <c r="L8" s="5">
+        <v>0.76770000000000005</v>
+      </c>
+      <c r="M8">
+        <v>460</v>
+      </c>
+      <c r="N8">
+        <v>13.3</v>
+      </c>
+      <c r="O8">
+        <v>0.76800000000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J4:J8">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4:K8">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>